<commit_message>
chore: actualiza reporte de cambios al 2026-06-20
</commit_message>
<xml_diff>
--- a/cambios_tinacode.xlsx
+++ b/cambios_tinacode.xlsx
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -595,7 +595,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Reporte de Cambios · TinaCode  —  2026-06-01 al 2026-06-19</t>
+          <t>Reporte de Cambios · TinaCode  —  2026-06-01 al 2026-06-20</t>
         </is>
       </c>
     </row>
@@ -664,6 +664,16 @@
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -714,6 +724,16 @@
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
@@ -732,6 +752,16 @@
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
@@ -750,6 +780,16 @@
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
@@ -800,6 +840,16 @@
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -822,6 +872,16 @@
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -844,6 +904,16 @@
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
@@ -866,6 +936,16 @@
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
@@ -888,6 +968,16 @@
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -910,6 +1000,16 @@
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -932,6 +1032,16 @@
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -954,6 +1064,16 @@
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -976,6 +1096,16 @@
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -998,6 +1128,16 @@
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1020,6 +1160,16 @@
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1042,6 +1192,16 @@
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1064,6 +1224,16 @@
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1086,6 +1256,16 @@
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1140,6 +1320,16 @@
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Vie</t>
+        </is>
+      </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1162,6 +1352,16 @@
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Vie</t>
+        </is>
+      </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1184,6 +1384,16 @@
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Vie</t>
+        </is>
+      </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1206,6 +1416,16 @@
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Vie</t>
+        </is>
+      </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1228,6 +1448,16 @@
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Vie</t>
+        </is>
+      </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1250,6 +1480,16 @@
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Vie</t>
+        </is>
+      </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1272,6 +1512,16 @@
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Vie</t>
+        </is>
+      </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1294,6 +1544,16 @@
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Vie</t>
+        </is>
+      </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1316,6 +1576,16 @@
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Vie</t>
+        </is>
+      </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1370,6 +1640,16 @@
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1392,6 +1672,16 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1414,6 +1704,16 @@
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1436,6 +1736,16 @@
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1458,6 +1768,16 @@
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1480,6 +1800,16 @@
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1502,6 +1832,16 @@
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1524,6 +1864,16 @@
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1546,6 +1896,16 @@
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1568,6 +1928,16 @@
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1590,6 +1960,16 @@
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1612,6 +1992,16 @@
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1634,6 +2024,16 @@
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1656,6 +2056,16 @@
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C48" s="14" t="inlineStr">
         <is>
           <t>Refactorización</t>
@@ -1678,6 +2088,16 @@
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1700,6 +2120,16 @@
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1722,6 +2152,16 @@
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1744,6 +2184,16 @@
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1766,6 +2216,16 @@
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1788,6 +2248,16 @@
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1842,6 +2312,16 @@
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -1864,6 +2344,16 @@
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
           <t>Rendimiento</t>
@@ -1886,6 +2376,16 @@
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1908,6 +2408,16 @@
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1930,6 +2440,16 @@
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1952,6 +2472,16 @@
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1974,6 +2504,16 @@
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -1996,6 +2536,16 @@
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -2050,6 +2600,16 @@
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="C65" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -2072,6 +2632,16 @@
       </c>
     </row>
     <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -2094,6 +2664,16 @@
       </c>
     </row>
     <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -2116,6 +2696,16 @@
       </c>
     </row>
     <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -2138,6 +2728,16 @@
       </c>
     </row>
     <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
@@ -2256,6 +2856,16 @@
       </c>
     </row>
     <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C73" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -2278,6 +2888,16 @@
       </c>
     </row>
     <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C74" s="12" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
@@ -2300,6 +2920,16 @@
       </c>
     </row>
     <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
           <t>Documentación</t>
@@ -2322,6 +2952,16 @@
       </c>
     </row>
     <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -2344,6 +2984,16 @@
       </c>
     </row>
     <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
       <c r="C77" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -2398,6 +3048,16 @@
       </c>
     </row>
     <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
       <c r="C79" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -2420,6 +3080,16 @@
       </c>
     </row>
     <row r="80" ht="18" customHeight="1">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -2442,6 +3112,16 @@
       </c>
     </row>
     <row r="81" ht="18" customHeight="1">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
       <c r="C81" s="12" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
@@ -2464,6 +3144,16 @@
       </c>
     </row>
     <row r="82" ht="18" customHeight="1">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
       <c r="C82" s="12" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
@@ -2514,6 +3204,16 @@
       </c>
     </row>
     <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
           <t>Corrección</t>
@@ -2546,316 +3246,510 @@
           <t>Jue</t>
         </is>
       </c>
-      <c r="C85" s="8" t="inlineStr">
+      <c r="C85" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>repite Fecha/Día por fila — elimina merge_cells incompatible con Google Sheets</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="inlineStr">
+        <is>
+          <t>REPORT</t>
+        </is>
+      </c>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="18" customHeight="1">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
         </is>
       </c>
-      <c r="D85" s="5" t="inlineStr">
+      <c r="D86" s="9" t="inlineStr">
         <is>
           <t>redistribuye cc-row — elimina cc-icon, nuevo cc-bottom con chip + botón</t>
         </is>
       </c>
-      <c r="E85" s="6" t="inlineStr">
+      <c r="E86" s="10" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="F85" s="7" t="inlineStr">
-        <is>
-          <t>Gerardo Herrera</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="18" customHeight="1">
-      <c r="C86" s="13" t="inlineStr">
-        <is>
-          <t>Corrección</t>
-        </is>
-      </c>
-      <c r="D86" s="9" t="inlineStr">
+      <c r="F86" s="11" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="C87" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
         <is>
           <t>ajusta pv-icon a translateY(10px)</t>
         </is>
       </c>
-      <c r="E86" s="10" t="inlineStr">
+      <c r="E87" s="6" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="F86" s="11" t="inlineStr">
-        <is>
-          <t>Gerardo Herrera</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="18" customHeight="1">
-      <c r="C87" s="13" t="inlineStr">
-        <is>
-          <t>Corrección</t>
-        </is>
-      </c>
-      <c r="D87" s="5" t="inlineStr">
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="C88" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D88" s="9" t="inlineStr">
         <is>
           <t>baja pv-icon 5px con translateY</t>
         </is>
       </c>
-      <c r="E87" s="6" t="inlineStr">
+      <c r="E88" s="10" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="F87" s="7" t="inlineStr">
-        <is>
-          <t>Gerardo Herrera</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="18" customHeight="1">
-      <c r="C88" s="13" t="inlineStr">
-        <is>
-          <t>Corrección</t>
-        </is>
-      </c>
-      <c r="D88" s="9" t="inlineStr">
+      <c r="F88" s="11" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="18" customHeight="1">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="C89" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
         <is>
           <t>regresa pv-icon al centro y reduce cc-preview a 125px</t>
         </is>
       </c>
-      <c r="E88" s="10" t="inlineStr">
+      <c r="E89" s="6" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="F88" s="11" t="inlineStr">
-        <is>
-          <t>Gerardo Herrera</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="18" customHeight="1">
-      <c r="C89" s="8" t="inlineStr">
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="18" customHeight="1">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
         <is>
           <t>Nueva función</t>
         </is>
       </c>
-      <c r="D89" s="5" t="inlineStr">
+      <c r="D90" s="9" t="inlineStr">
         <is>
           <t>redistribuye elementos de cc-preview en catalog-card</t>
         </is>
       </c>
-      <c r="E89" s="6" t="inlineStr">
+      <c r="E90" s="10" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="F89" s="7" t="inlineStr">
-        <is>
-          <t>Gerardo Herrera</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="18" customHeight="1">
-      <c r="C90" s="12" t="inlineStr">
+      <c r="F90" s="11" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="18" customHeight="1">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="C91" s="12" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="D90" s="9" t="inlineStr">
+      <c r="D91" s="5" t="inlineStr">
         <is>
           <t>acepta REPO y OUT como argumentos CLI en generate_report.py</t>
         </is>
       </c>
-      <c r="E90" s="10" t="inlineStr">
+      <c r="E91" s="6" t="inlineStr">
         <is>
           <t>REPORTS</t>
         </is>
       </c>
-      <c r="F90" s="11" t="inlineStr">
-        <is>
-          <t>Gerardo Herrera</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="18" customHeight="1">
-      <c r="C91" s="13" t="inlineStr">
-        <is>
-          <t>Corrección</t>
-        </is>
-      </c>
-      <c r="D91" s="5" t="inlineStr">
+      <c r="F91" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="18" customHeight="1">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="C92" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D92" s="9" t="inlineStr">
         <is>
           <t>extrae 13 estilos tipográficos inline a clases CSS</t>
         </is>
       </c>
-      <c r="E91" s="6" t="inlineStr">
+      <c r="E92" s="10" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="F91" s="7" t="inlineStr">
-        <is>
-          <t>Gerardo Herrera</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="18" customHeight="1">
-      <c r="C92" s="13" t="inlineStr">
-        <is>
-          <t>Corrección</t>
-        </is>
-      </c>
-      <c r="D92" s="9" t="inlineStr">
+      <c r="F92" s="11" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="C93" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
         <is>
           <t>agrega line-height explícito a 4 elementos de texto multilinea</t>
         </is>
       </c>
-      <c r="E92" s="10" t="inlineStr">
+      <c r="E93" s="6" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="F92" s="11" t="inlineStr">
-        <is>
-          <t>Gerardo Herrera</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="18" customHeight="1">
-      <c r="C93" s="13" t="inlineStr">
-        <is>
-          <t>Corrección</t>
-        </is>
-      </c>
-      <c r="D93" s="5" t="inlineStr">
+      <c r="F93" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="18" customHeight="1">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="C94" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D94" s="9" t="inlineStr">
         <is>
           <t>agrega font-family a .cat-explore-head .row-eyebrow</t>
         </is>
       </c>
-      <c r="E93" s="6" t="inlineStr">
+      <c r="E94" s="10" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="F93" s="7" t="inlineStr">
-        <is>
-          <t>Gerardo Herrera</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="18" customHeight="1">
-      <c r="C94" s="13" t="inlineStr">
-        <is>
-          <t>Corrección</t>
-        </is>
-      </c>
-      <c r="D94" s="9" t="inlineStr">
+      <c r="F94" s="11" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="18" customHeight="1">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="C95" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
         <is>
           <t>sube font-size de labels del gráfico analytics de 9px a 11px</t>
         </is>
       </c>
-      <c r="E94" s="10" t="inlineStr">
+      <c r="E95" s="6" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="F94" s="11" t="inlineStr">
-        <is>
-          <t>Gerardo Herrera</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="18" customHeight="1">
-      <c r="C95" s="13" t="inlineStr">
-        <is>
-          <t>Corrección</t>
-        </is>
-      </c>
-      <c r="D95" s="5" t="inlineStr">
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="18" customHeight="1">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="C96" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D96" s="9" t="inlineStr">
         <is>
           <t>corrige letter-spacing de .login-card h1 a -.02em</t>
         </is>
       </c>
-      <c r="E95" s="6" t="inlineStr">
+      <c r="E96" s="10" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="F95" s="7" t="inlineStr">
-        <is>
-          <t>Gerardo Herrera</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="18" customHeight="1">
-      <c r="C96" s="13" t="inlineStr">
-        <is>
-          <t>Corrección</t>
-        </is>
-      </c>
-      <c r="D96" s="9" t="inlineStr">
+      <c r="F96" s="11" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="18" customHeight="1">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="C97" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
         <is>
           <t>convierte letter-spacing de px a em en toda la hoja de estilos</t>
         </is>
       </c>
-      <c r="E96" s="10" t="inlineStr">
+      <c r="E97" s="6" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="F96" s="11" t="inlineStr">
-        <is>
-          <t>Gerardo Herrera</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="18" customHeight="1">
-      <c r="C97" s="13" t="inlineStr">
-        <is>
-          <t>Corrección</t>
-        </is>
-      </c>
-      <c r="D97" s="5" t="inlineStr">
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="18" customHeight="1">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="C98" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D98" s="9" t="inlineStr">
         <is>
           <t>elimina definiciones CSS conflictivas — unifica escala tipográfica</t>
         </is>
       </c>
-      <c r="E97" s="6" t="inlineStr">
+      <c r="E98" s="10" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="F97" s="7" t="inlineStr">
+      <c r="F98" s="11" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="18" customHeight="1">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>Vie</t>
+        </is>
+      </c>
+      <c r="C99" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>enriquece títulos consultando deploys de prod en QA</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t>WEEKLY-REPORT</t>
+        </is>
+      </c>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="18" customHeight="1">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>Vie</t>
+        </is>
+      </c>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>Nueva función</t>
+        </is>
+      </c>
+      <c r="D100" s="9" t="inlineStr">
+        <is>
+          <t>reporte semanal automático con opt-in por app</t>
+        </is>
+      </c>
+      <c r="E100" s="10" t="inlineStr">
+        <is>
+          <t>WEEKLY-REPORT</t>
+        </is>
+      </c>
+      <c r="F100" s="11" t="inlineStr">
         <is>
           <t>Gerardo Herrera</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="A9:A23"/>
-    <mergeCell ref="B78:B82"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="A64:A69"/>
-    <mergeCell ref="A55:A63"/>
-    <mergeCell ref="B72:B77"/>
-    <mergeCell ref="A34:A54"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A24:A33"/>
-    <mergeCell ref="A85:A97"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="B9:B23"/>
-    <mergeCell ref="B55:B63"/>
-    <mergeCell ref="A5:A8"/>
-    <mergeCell ref="B85:B97"/>
-    <mergeCell ref="B5:B8"/>
-    <mergeCell ref="A78:A82"/>
-    <mergeCell ref="B64:B69"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B34:B54"/>
-    <mergeCell ref="A83:A84"/>
-    <mergeCell ref="A72:A77"/>
-    <mergeCell ref="B24:B33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2896,7 +3790,7 @@
         </is>
       </c>
       <c r="B3" s="19" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
@@ -2911,11 +3805,11 @@
         </is>
       </c>
       <c r="B4" s="19" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>27%</t>
         </is>
       </c>
     </row>
@@ -2930,7 +3824,7 @@
       </c>
       <c r="C5" s="20" t="inlineStr">
         <is>
-          <t>11%</t>
+          <t>10%</t>
         </is>
       </c>
     </row>
@@ -2986,7 +3880,7 @@
         </is>
       </c>
       <c r="B10" s="19" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11">
@@ -2996,7 +3890,7 @@
         </is>
       </c>
       <c r="B11" s="19" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -3013,7 +3907,7 @@
         </is>
       </c>
       <c r="B14" s="19" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
chore: actualiza reporte de cambios al 2026-06-23
</commit_message>
<xml_diff>
--- a/cambios_tinacode.xlsx
+++ b/cambios_tinacode.xlsx
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -595,7 +595,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Reporte de Cambios · TinaCode  —  2026-06-01 al 2026-06-20</t>
+          <t>Reporte de Cambios · TinaCode  —  2026-06-01 al 2026-06-23</t>
         </is>
       </c>
     </row>
@@ -3742,6 +3742,390 @@
         </is>
       </c>
       <c r="F100" s="11" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="18" customHeight="1">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
+      <c r="C101" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>cambia etiqueta ESTE MES a estilo amb-lbl</t>
+        </is>
+      </c>
+      <c r="E101" s="6" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F101" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="18" customHeight="1">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
+      <c r="C102" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D102" s="9" t="inlineStr">
+        <is>
+          <t>cambia etiqueta TOP por Top User con estilo amb-lbl</t>
+        </is>
+      </c>
+      <c r="E102" s="10" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F102" s="11" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="18" customHeight="1">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
+      <c r="C103" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>texto este mes y Top en mayúsculas en banda de métricas</t>
+        </is>
+      </c>
+      <c r="E103" s="6" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F103" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="18" customHeight="1">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
+      <c r="C104" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D104" s="9" t="inlineStr">
+        <is>
+          <t>elimina bloque Tipo Acceso de la banda de métricas</t>
+        </is>
+      </c>
+      <c r="E104" s="10" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F104" s="11" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="18" customHeight="1">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
+      <c r="C105" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>separa datos de QA y prod en admin stats y share tokens</t>
+        </is>
+      </c>
+      <c r="E105" s="6" t="inlineStr">
+        <is>
+          <t>DATA-ISOLATION</t>
+        </is>
+      </c>
+      <c r="F105" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="18" customHeight="1">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
+      <c r="C106" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D106" s="9" t="inlineStr">
+        <is>
+          <t>corrige título de app eliminada en banda de métricas</t>
+        </is>
+      </c>
+      <c r="E106" s="10" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F106" s="11" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="18" customHeight="1">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
+      <c r="C107" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>corrige título de app con más aperturas en banda de métricas</t>
+        </is>
+      </c>
+      <c r="E107" s="6" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F107" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="18" customHeight="1">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>Nueva función</t>
+        </is>
+      </c>
+      <c r="D108" s="9" t="inlineStr">
+        <is>
+          <t>agrega bloque 'App con más aperturas' en la banda de métricas</t>
+        </is>
+      </c>
+      <c r="E108" s="10" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F108" s="11" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="18" customHeight="1">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
+      <c r="C109" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>ajusta etiquetas y elimina sección Salud de la banda de métricas</t>
+        </is>
+      </c>
+      <c r="E109" s="6" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F109" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="18" customHeight="1">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>Nueva función</t>
+        </is>
+      </c>
+      <c r="D110" s="9" t="inlineStr">
+        <is>
+          <t>banda de métricas secundaria en panel admin</t>
+        </is>
+      </c>
+      <c r="E110" s="10" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F110" s="11" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="18" customHeight="1">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
+      <c r="C111" s="13" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>agrega traducción th_health en los tres idiomas</t>
+        </is>
+      </c>
+      <c r="E111" s="6" t="inlineStr">
+        <is>
+          <t>HEALTH-MONITOR</t>
+        </is>
+      </c>
+      <c r="F111" s="7" t="inlineStr">
+        <is>
+          <t>Gerardo Herrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="18" customHeight="1">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>Lun</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="inlineStr">
+        <is>
+          <t>Nueva función</t>
+        </is>
+      </c>
+      <c r="D112" s="9" t="inlineStr">
+        <is>
+          <t>monitor automático de salud de apps publicadas</t>
+        </is>
+      </c>
+      <c r="E112" s="10" t="inlineStr">
+        <is>
+          <t>HEALTH-MONITOR</t>
+        </is>
+      </c>
+      <c r="F112" s="11" t="inlineStr">
         <is>
           <t>Gerardo Herrera</t>
         </is>
@@ -3790,11 +4174,11 @@
         </is>
       </c>
       <c r="B3" s="19" t="n">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
-          <t>59%</t>
+          <t>61%</t>
         </is>
       </c>
     </row>
@@ -3805,11 +4189,11 @@
         </is>
       </c>
       <c r="B4" s="19" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>26%</t>
         </is>
       </c>
     </row>
@@ -3824,7 +4208,7 @@
       </c>
       <c r="C5" s="20" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>9%</t>
         </is>
       </c>
     </row>
@@ -3880,7 +4264,7 @@
         </is>
       </c>
       <c r="B10" s="19" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11">
@@ -3890,7 +4274,7 @@
         </is>
       </c>
       <c r="B11" s="19" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -3907,7 +4291,7 @@
         </is>
       </c>
       <c r="B14" s="19" t="n">
-        <v>96</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15">

</xml_diff>